<commit_message>
[ADD] Updated SMOTE[NC] gridsearch models. Mean-based metric
</commit_message>
<xml_diff>
--- a/results/metrics_modelling4_smote_mean_opt.xlsx
+++ b/results/metrics_modelling4_smote_mean_opt.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DH8"/>
+  <dimension ref="A1:DH17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1073,31 +1073,31 @@
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>0.007159233093261719, 0.006227016448974609, 0.005711078643798828, 0.00559687614440918, 0.0060389041900634766, 0.005403757095336914, 0.005224943161010742</t>
+          <t>0.0067691802978515625, 0.005438089370727539, 0.005393028259277344, 0.005741119384765625, 0.005205869674682617, 0.0058138370513916016, 0.005396842956542969</t>
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>0.005908829825265067</v>
+        <v>0.005679709570748466</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.005711078643798828</v>
+        <v>0.005438089370727539</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.0006024818267958567</v>
+        <v>0.0004860646746321166</v>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>0.00837564468383789, 0.009192943572998047, 0.012052059173583984, 0.007241010665893555, 0.008144140243530273, 0.006852149963378906, 0.0074040889739990234</t>
+          <t>0.007107257843017578, 0.0065839290618896484, 0.006695985794067383, 0.006824970245361328, 0.0067403316497802734, 0.006675004959106445, 0.006965160369873047</t>
         </is>
       </c>
       <c r="AD2" t="n">
-        <v>0.008466005325317383</v>
+        <v>0.006798948560442243</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.008144140243530273</v>
+        <v>0.006740331649780273</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.001635882941021799</v>
+        <v>0.0001686038391138155</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
@@ -1463,31 +1463,31 @@
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>0.006283998489379883, 0.006273031234741211, 0.011313915252685547, 0.00483393669128418, 0.004912853240966797, 0.004408836364746094, 0.004515171051025391</t>
+          <t>0.007014036178588867, 0.004857778549194336, 0.004539012908935547, 0.005191802978515625, 0.007134914398193359, 0.004791736602783203, 0.005089998245239258</t>
         </is>
       </c>
       <c r="Z3" t="n">
-        <v>0.006077391760689872</v>
+        <v>0.005517039980207171</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.004912853240966797</v>
+        <v>0.005089998245239258</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.002256073724572875</v>
+        <v>0.001004552962187728</v>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>0.0062830448150634766, 0.021465063095092773, 0.007622957229614258, 0.0059719085693359375, 0.00577092170715332, 0.005928754806518555, 0.006413698196411133</t>
+          <t>0.008672714233398438, 0.007194042205810547, 0.0063991546630859375, 0.008219003677368164, 0.0067708492279052734, 0.0064661502838134766, 0.00656580924987793</t>
         </is>
       </c>
       <c r="AD3" t="n">
-        <v>0.008493764059884208</v>
+        <v>0.007183960505894252</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.006283044815063477</v>
+        <v>0.006770849227905273</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.00532621220052486</v>
+        <v>0.0008427630829421879</v>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
@@ -1853,31 +1853,31 @@
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>0.005089759826660156, 0.00453495979309082, 0.004294872283935547, 0.004211902618408203, 0.004590749740600586, 0.004415988922119141, 0.004103899002075195</t>
+          <t>0.0073451995849609375, 0.004645824432373047, 0.004674196243286133, 0.004609107971191406, 0.004503965377807617, 0.0045931339263916016, 0.004388093948364258</t>
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>0.004463161740984235</v>
+        <v>0.004965645926339286</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.004415988922119141</v>
+        <v>0.004609107971191406</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.0003016161935176782</v>
+        <v>0.0009755660656940003</v>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>0.008062124252319336, 0.008096933364868164, 0.008570194244384766, 0.007853984832763672, 0.007461071014404297, 0.007566928863525391, 0.008300065994262695</t>
+          <t>0.01160287857055664, 0.009387969970703125, 0.008130073547363281, 0.009238958358764648, 0.008074045181274414, 0.008416175842285156, 0.009328842163085938</t>
         </is>
       </c>
       <c r="AD4" t="n">
-        <v>0.007987328938075475</v>
+        <v>0.0091684205191476</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.008062124252319336</v>
+        <v>0.009238958358764648</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.0003638304503762481</v>
+        <v>0.001124226243386786</v>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
@@ -2243,31 +2243,31 @@
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>0.005602121353149414, 0.004238128662109375, 0.0036580562591552734, 0.0033910274505615234, 0.003653287887573242, 0.0038139820098876953, 0.003435850143432617</t>
+          <t>0.005604982376098633, 0.0041961669921875, 0.004109859466552734, 0.003693103790283203, 0.003904104232788086, 0.00416874885559082, 0.055033206939697266</t>
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>0.003970350537981305</v>
+        <v>0.01153002466474261</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.003658056259155273</v>
+        <v>0.00416874885559082</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.0007149619955769531</v>
+        <v>0.01776930614798336</v>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>0.007370948791503906, 0.0066907405853271484, 0.006968021392822266, 0.007401943206787109, 0.006975889205932617, 0.007158041000366211, 0.0066602230072021484</t>
+          <t>0.009300947189331055, 0.00962519645690918, 0.0114898681640625, 0.0073621273040771484, 0.007603883743286133, 0.01691126823425293, 0.019090890884399414</t>
         </is>
       </c>
       <c r="AD5" t="n">
-        <v>0.00703225816999163</v>
+        <v>0.01162631171090262</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.006975889205932617</v>
+        <v>0.00962519645690918</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.0002750449133673932</v>
+        <v>0.004266887496601929</v>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
@@ -2633,31 +2633,31 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>0.013518810272216797, 0.012042999267578125, 0.012275934219360352, 0.01221919059753418, 0.012650012969970703, 0.012105941772460938, 0.011887788772583008</t>
+          <t>0.014297008514404297, 0.014793872833251953, 0.01237797737121582, 0.012809991836547852, 0.013186931610107422, 0.012434959411621094, 0.012617111206054688</t>
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>0.01238581112452916</v>
+        <v>0.01321683611188616</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.01221919059753418</v>
+        <v>0.01280999183654785</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.0005123054480389144</v>
+        <v>0.0008859957196922687</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>0.007920265197753906, 0.007838010787963867, 0.007256984710693359, 0.00728607177734375, 0.00757288932800293, 0.007517337799072266, 0.0069272518157958984</t>
+          <t>0.007470846176147461, 0.007607936859130859, 0.007752895355224609, 0.008597135543823242, 0.007718086242675781, 0.0077860355377197266, 0.007859945297241211</t>
         </is>
       </c>
       <c r="AD6" t="n">
-        <v>0.007474115916660854</v>
+        <v>0.007827554430280412</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.007517337799072266</v>
+        <v>0.007752895355224609</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.0003217496542431411</v>
+        <v>0.0003355290055023129</v>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
@@ -3023,31 +3023,31 @@
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>0.011702775955200195, 0.009884834289550781, 0.010586023330688477, 0.010392189025878906, 0.010663986206054688, 0.010020017623901367, 0.010879993438720703</t>
+          <t>0.012148857116699219, 0.010150909423828125, 0.010843992233276367, 0.010285139083862305, 0.010724782943725586, 0.01074981689453125, 0.011121273040771484</t>
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>0.01058997426714216</v>
+        <v>0.01086068153381348</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.01058602333068848</v>
+        <v>0.01074981689453125</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.0005592244704769806</v>
+        <v>0.0006086715925960631</v>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>0.006797075271606445, 0.006165981292724609, 0.006516933441162109, 0.006468772888183594, 0.007037162780761719, 0.0063991546630859375, 0.006542205810546875</t>
+          <t>0.007092952728271484, 0.00698399543762207, 0.0067901611328125, 0.0066831111907958984, 0.006726264953613281, 0.006674289703369141, 0.0069158077239990234</t>
         </is>
       </c>
       <c r="AD7" t="n">
-        <v>0.006561040878295898</v>
+        <v>0.006838083267211914</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.006516933441162109</v>
+        <v>0.0067901611328125</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.0002606303160326355</v>
+        <v>0.0001502067323409855</v>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
@@ -3413,31 +3413,31 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>0.656606912612915, 0.6931262016296387, 0.63690185546875, 0.6366751194000244, 0.6457068920135498, 0.6470780372619629, 0.639066219329834</t>
+          <t>0.7405400276184082, 0.8228521347045898, 0.8180508613586426, 0.7622458934783936, 0.7943110466003418, 0.7523829936981201, 0.8533389568328857</t>
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>0.6507373196738107</v>
+        <v>0.7919602734701974</v>
       </c>
       <c r="AA8" t="n">
-        <v>0.6457068920135498</v>
+        <v>0.7943110466003418</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.01849843666946497</v>
+        <v>0.03873212381851463</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>0.007891178131103516, 0.008076667785644531, 0.007841110229492188, 0.007462978363037109, 0.007193803787231445, 0.007281064987182617, 0.008496761322021484</t>
+          <t>0.0075299739837646484, 0.008975744247436523, 0.009743213653564453, 0.008033990859985352, 0.007512807846069336, 0.007661104202270508, 0.008344173431396484</t>
         </is>
       </c>
       <c r="AD8" t="n">
-        <v>0.007749080657958984</v>
+        <v>0.008257286889212472</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.007841110229492188</v>
+        <v>0.008033990859985352</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.0004316457591864683</v>
+        <v>0.0007764605239532914</v>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
@@ -3718,6 +3718,3516 @@
       </c>
       <c r="DH8" t="n">
         <v>0.0002243620806489561</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CatBoostClassifier_no_fragmentation_smote_grid-opt-mean-smote_default-model</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>{'estimator': 'CatBoostClassifier', 'estimator_params': {'verbose': False}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {'k_neighbors': 7, 'sampling_strategy': 0.6}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.9854545454545455</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.8977272727272727</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.8977272727272727</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.9454545454545454</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.9454545454545454</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.9454545454545454</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.9932659932659933</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.9753086419753086</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.9875</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0.9998258042039252</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.9914458525345622</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.9954128440366973</v>
+      </c>
+      <c r="V9" t="n">
+        <v>1</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.9908256880733946</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0.9953917050691244</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>0.793179988861084, 0.7934577465057373, 0.8289229869842529, 0.7861411571502686, 0.7560877799987793, 0.792015790939331, 0.7635347843170166</t>
+        </is>
+      </c>
+      <c r="Z9" t="n">
+        <v>0.7876200335366386</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>0.7920157909393311</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.02193111931568551</v>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>0.007947921752929688, 0.007160186767578125, 0.00904393196105957, 0.0071871280670166016, 0.00747227668762207, 0.00908207893371582, 0.00846099853515625</t>
+        </is>
+      </c>
+      <c r="AD9" t="n">
+        <v>0.008050646100725447</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0.007947921752929688</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0.0007655534224082327</v>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>0.9074074074074074, 0.8490566037735849, 0.9245283018867925, 0.8867924528301887, 0.9622641509433962, 0.9433962264150944, 0.9433962264150944</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>0.8743589743589744, 0.8745421245421245, 0.88003663003663, 0.8772893772893773, 0.9285714285714286, 0.9157509157509157, 0.9386446886446886</t>
+        </is>
+      </c>
+      <c r="AI9" t="n">
+        <v>0.8984563055991629</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0.88003663003663</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.02607961172524965</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0.9166916242387941</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0.9245283018867925</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>0.03609351621237702</v>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>0.8275862068965518, 0.7647058823529412, 0.8461538461538461, 0.7999999999999999, 0.923076923076923, 0.888888888888889, 0.896551724137931</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>0.9367088607594937, 0.8888888888888888, 0.9500000000000001, 0.9210526315789475, 0.975, 0.9620253164556962, 0.9610389610389611</t>
+        </is>
+      </c>
+      <c r="AQ9" t="n">
+        <v>0.9421020941031409</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>0.9500000000000001</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0.02726588893481355</v>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>0.8821475338280227, 0.826797385620915, 0.8980769230769231, 0.8605263157894737, 0.9490384615384615, 0.9254571026722926, 0.9287953425884461</t>
+        </is>
+      </c>
+      <c r="AU9" t="n">
+        <v>0.8958341521592192</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>0.8980769230769231</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.03964076147827795</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>0.8495662102152975</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>0.0525229007147746</v>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>0.8571428571428571, 0.65, 0.9166666666666666, 0.75, 1.0, 0.9230769230769231, 0.8666666666666667</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>0.925, 0.9696969696969697, 0.926829268292683, 0.9459459459459459, 0.9512195121951219, 0.95, 0.9736842105263158</t>
+        </is>
+      </c>
+      <c r="BC9" t="n">
+        <v>0.9489108438081482</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>0.01740449033663503</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>0.8519361590790163</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>0.1086194131115752</v>
+      </c>
+      <c r="BI9" t="inlineStr">
+        <is>
+          <t>0.8, 0.9285714285714286, 0.7857142857142857, 0.8571428571428571, 0.8571428571428571, 0.8571428571428571, 0.9285714285714286</t>
+        </is>
+      </c>
+      <c r="BJ9" t="inlineStr">
+        <is>
+          <t>0.9487179487179487, 0.8205128205128205, 0.9743589743589743, 0.8974358974358975, 1.0, 0.9743589743589743, 0.9487179487179487</t>
+        </is>
+      </c>
+      <c r="BK9" t="n">
+        <v>0.9377289377289377</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>0.9487179487179487</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>0.05627213002101544</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>0.8591836734693877</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>0.05146742944048364</v>
+      </c>
+      <c r="BQ9" t="inlineStr">
+        <is>
+          <t>0.9692307692307692, 0.9084249084249084, 0.9853479853479854, 0.9304029304029304, 0.9945054945054945, 0.9120879120879121, 0.9871794871794872</t>
+        </is>
+      </c>
+      <c r="BR9" t="n">
+        <v>0.9553113553113554</v>
+      </c>
+      <c r="BS9" t="n">
+        <v>0.9692307692307692</v>
+      </c>
+      <c r="BT9" t="n">
+        <v>0.0345061944354013</v>
+      </c>
+      <c r="BU9" t="inlineStr">
+        <is>
+          <t>0.9937106918238994, 1.0, 0.9937304075235109, 0.9968652037617555, 0.9968652037617555, 0.9968652037617555, 0.9937304075235109</t>
+        </is>
+      </c>
+      <c r="BV9" t="inlineStr">
+        <is>
+          <t>0.9919108669108669, 1.0, 0.9919808949220714, 0.9941176470588236, 0.9978632478632479, 0.9978632478632479, 0.9919808949220714</t>
+        </is>
+      </c>
+      <c r="BW9" t="n">
+        <v>0.9951023999343328</v>
+      </c>
+      <c r="BX9" t="n">
+        <v>0.9941176470588236</v>
+      </c>
+      <c r="BY9" t="n">
+        <v>0.003159436146015735</v>
+      </c>
+      <c r="BZ9" t="n">
+        <v>0.9959667311651696</v>
+      </c>
+      <c r="CA9" t="n">
+        <v>0.9968652037617555</v>
+      </c>
+      <c r="CB9" t="n">
+        <v>0.00219678391174473</v>
+      </c>
+      <c r="CC9" t="inlineStr">
+        <is>
+          <t>0.9880952380952381, 1.0, 0.9882352941176471, 0.9940828402366864, 0.9941520467836257, 0.9941520467836257, 0.9882352941176471</t>
+        </is>
+      </c>
+      <c r="CD9" t="inlineStr">
+        <is>
+          <t>0.9957264957264957, 1.0, 0.9957264957264957, 0.9978678038379531, 0.9978586723768736, 0.9978586723768736, 0.9957264957264957</t>
+        </is>
+      </c>
+      <c r="CE9" t="n">
+        <v>0.9972520908244553</v>
+      </c>
+      <c r="CF9" t="n">
+        <v>0.9978586723768736</v>
+      </c>
+      <c r="CG9" t="n">
+        <v>0.001495149821458733</v>
+      </c>
+      <c r="CH9" t="inlineStr">
+        <is>
+          <t>0.9919108669108669, 1.0, 0.9919808949220714, 0.9959753220373198, 0.9960053595802496, 0.9960053595802496, 0.9919808949220714</t>
+        </is>
+      </c>
+      <c r="CI9" t="n">
+        <v>0.994836956850404</v>
+      </c>
+      <c r="CJ9" t="n">
+        <v>0.9959753220373198</v>
+      </c>
+      <c r="CK9" t="n">
+        <v>0.002817278361235357</v>
+      </c>
+      <c r="CL9" t="n">
+        <v>0.9924218228763528</v>
+      </c>
+      <c r="CM9" t="n">
+        <v>0.9940828402366864</v>
+      </c>
+      <c r="CN9" t="n">
+        <v>0.004139504433597427</v>
+      </c>
+      <c r="CO9" t="inlineStr">
+        <is>
+          <t>0.9880952380952381, 1.0, 0.9882352941176471, 1.0, 0.9883720930232558, 0.9883720930232558, 0.9882352941176471</t>
+        </is>
+      </c>
+      <c r="CP9" t="inlineStr">
+        <is>
+          <t>0.9957264957264957, 1.0, 0.9957264957264957, 0.9957446808510638, 1.0, 1.0, 0.9957264957264957</t>
+        </is>
+      </c>
+      <c r="CQ9" t="n">
+        <v>0.9975605954329358</v>
+      </c>
+      <c r="CR9" t="n">
+        <v>0.9957446808510638</v>
+      </c>
+      <c r="CS9" t="n">
+        <v>0.002112594711100439</v>
+      </c>
+      <c r="CT9" t="n">
+        <v>0.9916157160538634</v>
+      </c>
+      <c r="CU9" t="n">
+        <v>0.9883720930232558</v>
+      </c>
+      <c r="CV9" t="n">
+        <v>0.005303407062568835</v>
+      </c>
+      <c r="CW9" t="inlineStr">
+        <is>
+          <t>0.9880952380952381, 1.0, 0.9882352941176471, 0.9882352941176471, 1.0, 1.0, 0.9882352941176471</t>
+        </is>
+      </c>
+      <c r="CX9" t="inlineStr">
+        <is>
+          <t>0.9957264957264957, 1.0, 0.9957264957264957, 1.0, 0.9957264957264957, 0.9957264957264957, 0.9957264957264957</t>
+        </is>
+      </c>
+      <c r="CY9" t="n">
+        <v>0.996947496947497</v>
+      </c>
+      <c r="CZ9" t="n">
+        <v>0.9957264957264957</v>
+      </c>
+      <c r="DA9" t="n">
+        <v>0.001930572442105231</v>
+      </c>
+      <c r="DB9" t="n">
+        <v>0.9932573029211685</v>
+      </c>
+      <c r="DC9" t="n">
+        <v>0.9882352941176471</v>
+      </c>
+      <c r="DD9" t="n">
+        <v>0.005839526916084106</v>
+      </c>
+      <c r="DE9" t="inlineStr">
+        <is>
+          <t>0.9998982498982498, 1.0, 0.9999497234791352, 1.0, 1.0, 1.0, 0.9999497234791352</t>
+        </is>
+      </c>
+      <c r="DF9" t="n">
+        <v>0.9999710995509314</v>
+      </c>
+      <c r="DG9" t="n">
+        <v>1</v>
+      </c>
+      <c r="DH9" t="n">
+        <v>3.695922195409029e-05</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>XGBClassifier_splashing_smote_grid-opt-mean-smote_default-model</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>{'estimator': 'XGBClassifier', 'estimator_params': {}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {'k_neighbors': 7, 'sampling_strategy': 1.0}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.8979591836734694</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.9471450617283951</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.8528257456828885</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.8076923076923077</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.9948186528497409</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0.9974025974025974</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.9999751984126984</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0.996308954203691</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.9952380952380953</v>
+      </c>
+      <c r="V10" t="n">
+        <v>1</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0.9904761904761905</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0.9952153110047847</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>0.25836896896362305, 0.24454593658447266, 0.24982810020446777, 0.23743414878845215, 0.3201718330383301, 0.2678191661834717, 0.26900601387023926</t>
+        </is>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.2638820239475795</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0.258368968963623</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.02538722933165448</v>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>0.008426189422607422, 0.009593009948730469, 0.008414983749389648, 0.008800983428955078, 0.008508920669555664, 0.009994983673095703, 0.008940696716308594</t>
+        </is>
+      </c>
+      <c r="AD10" t="n">
+        <v>0.008954252515520369</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0.008800983428955078</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0.0005710628510154612</v>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>0.9629629629629629, 0.7924528301886793, 0.9245283018867925, 0.8301886792452831, 0.9056603773584906, 0.8301886792452831, 0.8679245283018868</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>0.9473684210526316, 0.8023809523809524, 0.9295665634674922, 0.8328173374613003, 0.903250773993808, 0.8560371517027863, 0.8390092879256965</t>
+        </is>
+      </c>
+      <c r="AI10" t="n">
+        <v>0.8729186411406668</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0.8560371517027863</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0.05027112793891122</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0.8734151941699111</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>0.05605255122691098</v>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>0.9722222222222222, 0.8307692307692307, 0.9393939393939394, 0.8615384615384616, 0.9253731343283583, 0.8524590163934426, 0.9014084507042254</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.7317073170731708, 0.9, 0.7804878048780488, 0.8717948717948718, 0.7999999999999999, 0.7999999999999999</t>
+        </is>
+      </c>
+      <c r="AQ10" t="n">
+        <v>0.8326334911700766</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>0.7999999999999999</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>0.06929100562647317</v>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>0.9583333333333333, 0.7812382739212007, 0.9196969696969697, 0.8210131332082552, 0.898584003061615, 0.8262295081967213, 0.8507042253521127</t>
+        </is>
+      </c>
+      <c r="AU10" t="n">
+        <v>0.8651142066814581</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>0.8507042253521127</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0.05792736212327599</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>0.89759492219284</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>0.9014084507042254</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>0.04766783161975097</v>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>0.9459459459459459, 0.9, 0.96875, 0.9032258064516129, 0.9393939393939394, 0.9629629629629629, 0.8648648648648649</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>1.0, 0.6521739130434783, 0.8571428571428571, 0.7272727272727273, 0.85, 0.6923076923076923, 0.875</t>
+        </is>
+      </c>
+      <c r="BC10" t="n">
+        <v>0.8076995985381078</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>0.1132095154495363</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>0.9264490742313323</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>0.9393939393939394</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>0.0352578632957699</v>
+      </c>
+      <c r="BI10" t="inlineStr">
+        <is>
+          <t>1.0, 0.7714285714285715, 0.9117647058823529, 0.8235294117647058, 0.9117647058823529, 0.7647058823529411, 0.9411764705882353</t>
+        </is>
+      </c>
+      <c r="BJ10" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.8333333333333334, 0.9473684210526315, 0.8421052631578947, 0.8947368421052632, 0.9473684210526315, 0.7368421052631579</t>
+        </is>
+      </c>
+      <c r="BK10" t="n">
+        <v>0.8709273182957393</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>0.06870551459585363</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>0.8749099639855943</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>0.9117647058823529</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>0.08302203697858708</v>
+      </c>
+      <c r="BQ10" t="inlineStr">
+        <is>
+          <t>0.9894736842105264, 0.946031746031746, 0.9752321981424148, 0.9489164086687307, 0.9442724458204335, 0.9303405572755418, 0.93343653250774</t>
+        </is>
+      </c>
+      <c r="BR10" t="n">
+        <v>0.9525290818081619</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>0.946031746031746</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>0.02021537609599209</v>
+      </c>
+      <c r="BU10" t="inlineStr">
+        <is>
+          <t>0.9968553459119497, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9968652037617555, 1.0, 0.9968652037617555</t>
+        </is>
+      </c>
+      <c r="BV10" t="inlineStr">
+        <is>
+          <t>0.995575221238938, 1.0, 0.995575221238938, 0.995575221238938, 0.995575221238938, 1.0, 0.995575221238938</t>
+        </is>
+      </c>
+      <c r="BW10" t="n">
+        <v>0.9968394437420985</v>
+      </c>
+      <c r="BX10" t="n">
+        <v>0.995575221238938</v>
+      </c>
+      <c r="BY10" t="n">
+        <v>0.001998911289613391</v>
+      </c>
+      <c r="BZ10" t="n">
+        <v>0.9977594515655674</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>0.9968652037617555</v>
+      </c>
+      <c r="CB10" t="n">
+        <v>0.001417051170840857</v>
+      </c>
+      <c r="CC10" t="inlineStr">
+        <is>
+          <t>0.9975669099756691, 1.0, 0.9975786924939467, 0.9975786924939467, 0.9975786924939467, 1.0, 0.9975786924939467</t>
+        </is>
+      </c>
+      <c r="CD10" t="inlineStr">
+        <is>
+          <t>0.9955555555555555, 1.0, 0.9955555555555555, 0.9955555555555555, 0.9955555555555555, 1.0, 0.9955555555555555</t>
+        </is>
+      </c>
+      <c r="CE10" t="n">
+        <v>0.9968253968253968</v>
+      </c>
+      <c r="CF10" t="n">
+        <v>0.9955555555555555</v>
+      </c>
+      <c r="CG10" t="n">
+        <v>0.00200779533978946</v>
+      </c>
+      <c r="CH10" t="inlineStr">
+        <is>
+          <t>0.9965612327656124, 1.0, 0.9965671240247511, 0.9965671240247511, 0.9965671240247511, 1.0, 0.9965671240247511</t>
+        </is>
+      </c>
+      <c r="CI10" t="n">
+        <v>0.9975471041235167</v>
+      </c>
+      <c r="CJ10" t="n">
+        <v>0.9965671240247511</v>
+      </c>
+      <c r="CK10" t="n">
+        <v>0.001551348844990803</v>
+      </c>
+      <c r="CL10" t="n">
+        <v>0.9982688114216364</v>
+      </c>
+      <c r="CM10" t="n">
+        <v>0.9975786924939467</v>
+      </c>
+      <c r="CN10" t="n">
+        <v>0.001094907038779773</v>
+      </c>
+      <c r="CO10" t="inlineStr">
+        <is>
+          <t>0.9951456310679612, 1.0, 0.9951690821256038, 0.9951690821256038, 0.9951690821256038, 1.0, 0.9951690821256038</t>
+        </is>
+      </c>
+      <c r="CP10" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CQ10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT10" t="n">
+        <v>0.9965459942243395</v>
+      </c>
+      <c r="CU10" t="n">
+        <v>0.9951690821256038</v>
+      </c>
+      <c r="CV10" t="n">
+        <v>0.002184519446236978</v>
+      </c>
+      <c r="CW10" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CX10" t="inlineStr">
+        <is>
+          <t>0.9911504424778761, 1.0, 0.9911504424778761, 0.9911504424778761, 0.9911504424778761, 1.0, 0.9911504424778761</t>
+        </is>
+      </c>
+      <c r="CY10" t="n">
+        <v>0.9936788874841972</v>
+      </c>
+      <c r="CZ10" t="n">
+        <v>0.9911504424778761</v>
+      </c>
+      <c r="DA10" t="n">
+        <v>0.003997822579226782</v>
+      </c>
+      <c r="DB10" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC10" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE10" t="inlineStr">
+        <is>
+          <t>0.9999784157133608, 1.0, 0.9999785204914512, 0.9999785204914512, 0.9999785204914512, 1.0, 0.9999785204914511</t>
+        </is>
+      </c>
+      <c r="DF10" t="n">
+        <v>0.999984642525595</v>
+      </c>
+      <c r="DG10" t="n">
+        <v>0.9999785204914512</v>
+      </c>
+      <c r="DH10" t="n">
+        <v>9.712984233443494e-06</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>XGBClassifier_no_fragmentation_smote_grid-opt-mean-smote_default-model</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>{'estimator': 'XGBClassifier', 'estimator_params': {}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {'k_neighbors': 8, 'sampling_strategy': 0.9}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.9066666666666666</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.8095238095238095</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.8292682926829269</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.9818181818181818</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.8825240545983442</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.8886363636363637</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.9272727272727272</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.9357798165137615</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="n">
+        <v>1</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1</v>
+      </c>
+      <c r="U11" t="n">
+        <v>1</v>
+      </c>
+      <c r="V11" t="n">
+        <v>1</v>
+      </c>
+      <c r="W11" t="n">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>0.22781109809875488, 0.24125099182128906, 0.2810487747192383, 0.24719500541687012, 0.24962806701660156, 0.2490081787109375, 0.3338658809661865</t>
+        </is>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.2614011423928397</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0.2490081787109375</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.03309184754304973</v>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>0.00776982307434082, 0.008003950119018555, 0.007461071014404297, 0.007875919342041016, 0.007687091827392578, 0.00847482681274414, 0.01051020622253418</t>
+        </is>
+      </c>
+      <c r="AD11" t="n">
+        <v>0.008254698344639369</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>0.007875919342041016</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0.0009657895408599467</v>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>0.8888888888888888, 0.8490566037735849, 0.9056603773584906, 0.8301886792452831, 0.9433962264150944, 0.9056603773584906, 0.9433962264150944</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>0.8410256410256409, 0.8287545787545787, 0.8672161172161172, 0.8388278388278387, 0.9157509157509157, 0.8672161172161172, 0.9615384615384616</t>
+        </is>
+      </c>
+      <c r="AI11" t="n">
+        <v>0.8743328100470958</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>0.8672161172161172</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0.04451151604293877</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0.8951781970649896</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>0.9056603773584906</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>0.04010718337465197</v>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>0.7857142857142856, 0.7333333333333334, 0.8148148148148148, 0.7272727272727273, 0.888888888888889, 0.8148148148148148, 0.9032258064516129</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>0.9249999999999999, 0.8947368421052632, 0.9367088607594937, 0.8767123287671232, 0.9620253164556962, 0.9367088607594937, 0.9600000000000001</t>
+        </is>
+      </c>
+      <c r="AQ11" t="n">
+        <v>0.9274131726924385</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>0.9367088607594937</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0.02946393194827078</v>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>0.8553571428571427, 0.8140350877192983, 0.8757618377871542, 0.8019925280199253, 0.9254571026722926, 0.8757618377871542, 0.9316129032258065</t>
+        </is>
+      </c>
+      <c r="AU11" t="n">
+        <v>0.8685683485812534</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>0.8757618377871542</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>0.04612899795543637</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>0.8097235244700682</v>
+      </c>
+      <c r="AY11" t="n">
+        <v>0.8148148148148148</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>0.06355168081410603</v>
+      </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>0.8461538461538461, 0.6875, 0.8461538461538461, 0.631578947368421, 0.9230769230769231, 0.8461538461538461, 0.8235294117647058</t>
+        </is>
+      </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>0.9024390243902439, 0.918918918918919, 0.925, 0.9411764705882353, 0.95, 0.925, 1.0</t>
+        </is>
+      </c>
+      <c r="BC11" t="n">
+        <v>0.9375049162710569</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>0.02918670159910827</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>0.8005924029530841</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>0.09495227307681021</v>
+      </c>
+      <c r="BI11" t="inlineStr">
+        <is>
+          <t>0.7333333333333333, 0.7857142857142857, 0.7857142857142857, 0.8571428571428571, 0.8571428571428571, 0.7857142857142857, 1.0</t>
+        </is>
+      </c>
+      <c r="BJ11" t="inlineStr">
+        <is>
+          <t>0.9487179487179487, 0.8717948717948718, 0.9487179487179487, 0.8205128205128205, 0.9743589743589743, 0.9487179487179487, 0.9230769230769231</t>
+        </is>
+      </c>
+      <c r="BK11" t="n">
+        <v>0.9194139194139195</v>
+      </c>
+      <c r="BL11" t="n">
+        <v>0.9487179487179487</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>0.05022457582711388</v>
+      </c>
+      <c r="BN11" t="n">
+        <v>0.8292517006802721</v>
+      </c>
+      <c r="BO11" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>0.08070906095218444</v>
+      </c>
+      <c r="BQ11" t="inlineStr">
+        <is>
+          <t>0.976068376068376, 0.9102564102564101, 0.9761904761904762, 0.9340659340659341, 0.9963369963369964, 0.923076923076923, 0.9926739926739927</t>
+        </is>
+      </c>
+      <c r="BR11" t="n">
+        <v>0.9583813012384441</v>
+      </c>
+      <c r="BS11" t="n">
+        <v>0.976068376068376</v>
+      </c>
+      <c r="BT11" t="n">
+        <v>0.0325143136281283</v>
+      </c>
+      <c r="BU11" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BV11" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BW11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC11" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CD11" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CE11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH11" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CI11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO11" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CP11" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CQ11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CU11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW11" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CX11" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CY11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ11" t="n">
+        <v>1</v>
+      </c>
+      <c r="DA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB11" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC11" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE11" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="DF11" t="n">
+        <v>1</v>
+      </c>
+      <c r="DG11" t="n">
+        <v>1</v>
+      </c>
+      <c r="DH11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>AdaBoostClassifier_splashing_smote_grid-opt-mean-smote_default-model</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>{'estimator': 'AdaBoostClassifier', 'estimator_params': {}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {'k_neighbors': 10, 'sampling_strategy': 0.9}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.851063829787234</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.8591820987654321</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.784688995215311</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.787037037037037</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.7142857142857143</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.7407407407407407</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.7272727272727273</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.9427609427609428</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.9629629629629629</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.9479166666666666</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0.9553805774278215</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.9932539682539682</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0.9377841854275257</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0.940625</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0.9074074074074074</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0.9201877934272301</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>0.04421710968017578, 0.03908491134643555, 0.03708004951477051, 0.10230708122253418, 0.034369707107543945, 0.03495287895202637, 0.03665900230407715</t>
+        </is>
+      </c>
+      <c r="Z12" t="n">
+        <v>0.04695296287536621</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0.03708004951477051</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>0.02280115889258556</v>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>0.010421991348266602, 0.011258840560913086, 0.018460750579833984, 0.011870861053466797, 0.010409355163574219, 0.012333869934082031, 0.011394023895263672</t>
+        </is>
+      </c>
+      <c r="AD12" t="n">
+        <v>0.01230709893362863</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>0.01139402389526367</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>0.002595217095907184</v>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>0.9074074074074074, 0.8301886792452831, 0.8490566037735849, 0.7924528301886793, 0.9056603773584906, 0.8113207547169812, 0.7547169811320755</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>0.868421052631579, 0.8174603174603174, 0.8243034055727554, 0.7801857585139318, 0.903250773993808, 0.8297213622291022, 0.7275541795665634</t>
+        </is>
+      </c>
+      <c r="AI12" t="n">
+        <v>0.8215566928525794</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>0.8243034055727554</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>0.05279232137251848</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>0.8358290905460716</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>0.8301886792452831</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>0.05246492459552389</v>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>0.9333333333333333, 0.8695652173913043, 0.8857142857142858, 0.8358208955223881, 0.9253731343283583, 0.8387096774193549, 0.8115942028985507</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>0.8484848484848484, 0.7567567567567567, 0.7777777777777778, 0.717948717948718, 0.8717948717948718, 0.7727272727272727, 0.6486486486486486</t>
+        </is>
+      </c>
+      <c r="AQ12" t="n">
+        <v>0.7705912705912705</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>0.7727272727272727</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>0.06989627205704758</v>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>0.8909090909090909, 0.8131609870740305, 0.8317460317460318, 0.776884806735553, 0.898584003061615, 0.8057184750733137, 0.7301214257735996</t>
+        </is>
+      </c>
+      <c r="AU12" t="n">
+        <v>0.8210178314818907</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>0.8131609870740305</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>0.05544891362232967</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>0.8714443923725108</v>
+      </c>
+      <c r="AY12" t="n">
+        <v>0.8695652173913043</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>0.04287582010502988</v>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>0.875, 0.8823529411764706, 0.8611111111111112, 0.8484848484848485, 0.9393939393939394, 0.9285714285714286, 0.8</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>1.0, 0.7368421052631579, 0.8235294117647058, 0.7, 0.85, 0.68, 0.6666666666666666</t>
+        </is>
+      </c>
+      <c r="BC12" t="n">
+        <v>0.7795768833849329</v>
+      </c>
+      <c r="BD12" t="n">
+        <v>0.7368421052631579</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>0.1110344893763404</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>0.8764163241053998</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>0.04404130498007724</v>
+      </c>
+      <c r="BI12" t="inlineStr">
+        <is>
+          <t>1.0, 0.8571428571428571, 0.9117647058823529, 0.8235294117647058, 0.9117647058823529, 0.7647058823529411, 0.8235294117647058</t>
+        </is>
+      </c>
+      <c r="BJ12" t="inlineStr">
+        <is>
+          <t>0.7368421052631579, 0.7777777777777778, 0.7368421052631579, 0.7368421052631579, 0.8947368421052632, 0.8947368421052632, 0.631578947368421</t>
+        </is>
+      </c>
+      <c r="BK12" t="n">
+        <v>0.772765246449457</v>
+      </c>
+      <c r="BL12" t="n">
+        <v>0.7368421052631579</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>0.08749224702814402</v>
+      </c>
+      <c r="BN12" t="n">
+        <v>0.8703481392557022</v>
+      </c>
+      <c r="BO12" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>0.07167278960035725</v>
+      </c>
+      <c r="BQ12" t="inlineStr">
+        <is>
+          <t>0.9383458646616541, 0.8873015873015874, 0.913312693498452, 0.9024767801857586, 0.9427244582043344, 0.8119195046439629, 0.8622291021671827</t>
+        </is>
+      </c>
+      <c r="BR12" t="n">
+        <v>0.8940442843804188</v>
+      </c>
+      <c r="BS12" t="n">
+        <v>0.9024767801857586</v>
+      </c>
+      <c r="BT12" t="n">
+        <v>0.04238752704731504</v>
+      </c>
+      <c r="BU12" t="inlineStr">
+        <is>
+          <t>0.9182389937106918, 0.9216300940438872, 0.9090909090909091, 0.9341692789968652, 0.9278996865203761, 0.9592476489028213, 0.9028213166144201</t>
+        </is>
+      </c>
+      <c r="BV12" t="inlineStr">
+        <is>
+          <t>0.9167278221454781, 0.9215019255455712, 0.9076381132399691, 0.929053183263167, 0.9301915972162558, 0.958458630466535, 0.8987885557178452</t>
+        </is>
+      </c>
+      <c r="BW12" t="n">
+        <v>0.9231942610849746</v>
+      </c>
+      <c r="BX12" t="n">
+        <v>0.9215019255455712</v>
+      </c>
+      <c r="BY12" t="n">
+        <v>0.0177650397140095</v>
+      </c>
+      <c r="BZ12" t="n">
+        <v>0.9247282754114244</v>
+      </c>
+      <c r="CA12" t="n">
+        <v>0.9216300940438872</v>
+      </c>
+      <c r="CB12" t="n">
+        <v>0.01718358484681609</v>
+      </c>
+      <c r="CC12" t="inlineStr">
+        <is>
+          <t>0.9356435643564357, 0.9379652605459058, 0.928395061728395, 0.9489051094890512, 0.9429280397022333, 0.9682151589242055, 0.9238329238329238</t>
+        </is>
+      </c>
+      <c r="CD12" t="inlineStr">
+        <is>
+          <t>0.8879310344827587, 0.8936170212765957, 0.8755364806866952, 0.9074889867841409, 0.902127659574468, 0.943231441048035, 0.8658008658008658</t>
+        </is>
+      </c>
+      <c r="CE12" t="n">
+        <v>0.8965333556647943</v>
+      </c>
+      <c r="CF12" t="n">
+        <v>0.8936170212765957</v>
+      </c>
+      <c r="CG12" t="n">
+        <v>0.02329896654968231</v>
+      </c>
+      <c r="CH12" t="inlineStr">
+        <is>
+          <t>0.9117872994195972, 0.9157911409112507, 0.9019657712075451, 0.928197048136596, 0.9225278496383507, 0.9557232999861203, 0.8948168948168949</t>
+        </is>
+      </c>
+      <c r="CI12" t="n">
+        <v>0.9186870434451935</v>
+      </c>
+      <c r="CJ12" t="n">
+        <v>0.9157911409112507</v>
+      </c>
+      <c r="CK12" t="n">
+        <v>0.01844781806647643</v>
+      </c>
+      <c r="CL12" t="n">
+        <v>0.9408407312255929</v>
+      </c>
+      <c r="CM12" t="n">
+        <v>0.9379652605459058</v>
+      </c>
+      <c r="CN12" t="n">
+        <v>0.01361820956301094</v>
+      </c>
+      <c r="CO12" t="inlineStr">
+        <is>
+          <t>0.949748743718593, 0.9545454545454546, 0.9447236180904522, 0.9512195121951219, 0.9644670050761421, 0.9753694581280788, 0.9353233830845771</t>
+        </is>
+      </c>
+      <c r="CP12" t="inlineStr">
+        <is>
+          <t>0.865546218487395, 0.8677685950413223, 0.85, 0.9035087719298246, 0.8688524590163934, 0.9310344827586207, 0.847457627118644</t>
+        </is>
+      </c>
+      <c r="CQ12" t="n">
+        <v>0.8763097363360287</v>
+      </c>
+      <c r="CR12" t="n">
+        <v>0.8677685950413223</v>
+      </c>
+      <c r="CS12" t="n">
+        <v>0.02803988800856164</v>
+      </c>
+      <c r="CT12" t="n">
+        <v>0.9536281678340599</v>
+      </c>
+      <c r="CU12" t="n">
+        <v>0.9512195121951219</v>
+      </c>
+      <c r="CV12" t="n">
+        <v>0.01210792665768993</v>
+      </c>
+      <c r="CW12" t="inlineStr">
+        <is>
+          <t>0.9219512195121952, 0.9219512195121952, 0.912621359223301, 0.9466019417475728, 0.9223300970873787, 0.9611650485436893, 0.912621359223301</t>
+        </is>
+      </c>
+      <c r="CX12" t="inlineStr">
+        <is>
+          <t>0.911504424778761, 0.9210526315789473, 0.9026548672566371, 0.911504424778761, 0.9380530973451328, 0.9557522123893806, 0.8849557522123894</t>
+        </is>
+      </c>
+      <c r="CY12" t="n">
+        <v>0.9179253443342869</v>
+      </c>
+      <c r="CZ12" t="n">
+        <v>0.911504424778761</v>
+      </c>
+      <c r="DA12" t="n">
+        <v>0.02154203931311345</v>
+      </c>
+      <c r="DB12" t="n">
+        <v>0.9284631778356618</v>
+      </c>
+      <c r="DC12" t="n">
+        <v>0.9219512195121952</v>
+      </c>
+      <c r="DD12" t="n">
+        <v>0.01699907316729176</v>
+      </c>
+      <c r="DE12" t="inlineStr">
+        <is>
+          <t>0.9798834448521476, 0.9839109970047069, 0.9804966062376492, 0.9862316350201907, 0.9817638972420311, 0.9926110490591975, 0.981248389036859</t>
+        </is>
+      </c>
+      <c r="DF12" t="n">
+        <v>0.9837351454932545</v>
+      </c>
+      <c r="DG12" t="n">
+        <v>0.9817638972420311</v>
+      </c>
+      <c r="DH12" t="n">
+        <v>0.004147952326222077</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>AdaBoostClassifier_no_fragmentation_smote_grid-opt-mean-smote_default-model</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>{'estimator': 'AdaBoostClassifier', 'estimator_params': {}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {'k_neighbors': 6, 'sampling_strategy': 0.6}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.7391304347826086</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.7906976744186046</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.9490909090909091</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.8532927624429472</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.8704545454545454</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.9423076923076923</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.8909090909090909</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.9158878504672897</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.9730639730639731</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.9176470588235294</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0.9873417721518988</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0.9512195121951219</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0.9958193008942051</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0.9663074305161656</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0.9776158402043897</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0.9952830188679245</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.9678899082568807</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0.9813953488372092</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>0.06338882446289062, 0.032479047775268555, 0.032704830169677734, 0.03319716453552246, 0.033941030502319336, 0.03191208839416504, 0.03241300582885742</t>
+        </is>
+      </c>
+      <c r="Z13" t="n">
+        <v>0.03714799880981445</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>0.03270483016967773</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>0.01072946833912126</v>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>0.040789127349853516, 0.010082721710205078, 0.009205102920532227, 0.00997304916381836, 0.009591102600097656, 0.013094186782836914, 0.009294986724853516</t>
+        </is>
+      </c>
+      <c r="AD13" t="n">
+        <v>0.01457575389317104</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>0.009973049163818359</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>0.01077222195128435</v>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>0.8148148148148148, 0.8301886792452831, 0.9245283018867925, 0.8301886792452831, 0.8867924528301887, 0.9056603773584906, 0.9245283018867925</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>0.7897435897435897, 0.8388278388278387, 0.88003663003663, 0.8388278388278387, 0.8543956043956045, 0.8672161172161172, 0.9029304029304028</t>
+        </is>
+      </c>
+      <c r="AI13" t="n">
+        <v>0.8531397174254316</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>0.8543956043956045</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>0.03344720209792343</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>0.8738145153239492</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>0.8867924528301887</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>0.04410013588092931</v>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>0.6875, 0.7272727272727273, 0.8461538461538461, 0.7272727272727273, 0.7857142857142857, 0.8148148148148148, 0.8571428571428571</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>0.868421052631579, 0.8767123287671232, 0.9500000000000001, 0.8767123287671232, 0.9230769230769231, 0.9367088607594937, 0.9487179487179487</t>
+        </is>
+      </c>
+      <c r="AQ13" t="n">
+        <v>0.9114784918171701</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>0.03362204660054285</v>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>0.7779605263157895, 0.8019925280199253, 0.8980769230769231, 0.8019925280199253, 0.8543956043956045, 0.8757618377871542, 0.9029304029304028</t>
+        </is>
+      </c>
+      <c r="AU13" t="n">
+        <v>0.8447300500779608</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>0.8543956043956045</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>0.0469052625837614</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>0.7779816083387512</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>0.06054530700835218</v>
+      </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>0.6470588235294118, 0.631578947368421, 0.9166666666666666, 0.631578947368421, 0.7857142857142857, 0.8461538461538461, 0.8571428571428571</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>0.8918918918918919, 0.9411764705882353, 0.926829268292683, 0.9411764705882353, 0.9230769230769231, 0.925, 0.9487179487179487</t>
+        </is>
+      </c>
+      <c r="BC13" t="n">
+        <v>0.928266996165131</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>0.926829268292683</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>0.01737969223386602</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>0.759413481991987</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>0.1119962522792415</v>
+      </c>
+      <c r="BI13" t="inlineStr">
+        <is>
+          <t>0.7333333333333333, 0.8571428571428571, 0.7857142857142857, 0.8571428571428571, 0.7857142857142857, 0.7857142857142857, 0.8571428571428571</t>
+        </is>
+      </c>
+      <c r="BJ13" t="inlineStr">
+        <is>
+          <t>0.8461538461538461, 0.8205128205128205, 0.9743589743589743, 0.8205128205128205, 0.9230769230769231, 0.9487179487179487, 0.9487179487179487</t>
+        </is>
+      </c>
+      <c r="BK13" t="n">
+        <v>0.8974358974358976</v>
+      </c>
+      <c r="BL13" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="BM13" t="n">
+        <v>0.06129377483766121</v>
+      </c>
+      <c r="BN13" t="n">
+        <v>0.808843537414966</v>
+      </c>
+      <c r="BO13" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>0.04520611626077863</v>
+      </c>
+      <c r="BQ13" t="inlineStr">
+        <is>
+          <t>0.8615384615384615, 0.9084249084249084, 0.9816849816849818, 0.9258241758241759, 0.9285714285714286, 0.923992673992674, 0.9780219780219781</t>
+        </is>
+      </c>
+      <c r="BR13" t="n">
+        <v>0.929722658294087</v>
+      </c>
+      <c r="BS13" t="n">
+        <v>0.9258241758241759</v>
+      </c>
+      <c r="BT13" t="n">
+        <v>0.03814435436712547</v>
+      </c>
+      <c r="BU13" t="inlineStr">
+        <is>
+          <t>0.9779874213836478, 0.9655172413793104, 0.9592476489028213, 0.9811912225705329, 0.9623824451410659, 0.9655172413793104, 0.9435736677115988</t>
+        </is>
+      </c>
+      <c r="BV13" t="inlineStr">
+        <is>
+          <t>0.9774114774114774, 0.9652589240824535, 0.9609854198089492, 0.9796882855706385, 0.959376571141277, 0.9652589240824535, 0.9428104575163399</t>
+        </is>
+      </c>
+      <c r="BW13" t="n">
+        <v>0.9643985799447984</v>
+      </c>
+      <c r="BX13" t="n">
+        <v>0.9652589240824535</v>
+      </c>
+      <c r="BY13" t="n">
+        <v>0.01138613346635316</v>
+      </c>
+      <c r="BZ13" t="n">
+        <v>0.9650595554954696</v>
+      </c>
+      <c r="CA13" t="n">
+        <v>0.9655172413793104</v>
+      </c>
+      <c r="CB13" t="n">
+        <v>0.01152864695153742</v>
+      </c>
+      <c r="CC13" t="inlineStr">
+        <is>
+          <t>0.95906432748538, 0.9371428571428572, 0.9265536723163841, 0.9651162790697674, 0.9310344827586207, 0.9371428571428572, 0.898876404494382</t>
+        </is>
+      </c>
+      <c r="CD13" t="inlineStr">
+        <is>
+          <t>0.9849462365591398, 0.9762419006479482, 0.9718004338394794, 0.9871244635193134, 0.9741379310344828, 0.9762419006479482, 0.9608695652173912</t>
+        </is>
+      </c>
+      <c r="CE13" t="n">
+        <v>0.9759089187808146</v>
+      </c>
+      <c r="CF13" t="n">
+        <v>0.9762419006479482</v>
+      </c>
+      <c r="CG13" t="n">
+        <v>0.008052342267687191</v>
+      </c>
+      <c r="CH13" t="inlineStr">
+        <is>
+          <t>0.9720052820222599, 0.9566923788954027, 0.9491770530779318, 0.9761203712945403, 0.9525862068965517, 0.9566923788954027, 0.9298729848558867</t>
+        </is>
+      </c>
+      <c r="CI13" t="n">
+        <v>0.9561638079911395</v>
+      </c>
+      <c r="CJ13" t="n">
+        <v>0.9566923788954027</v>
+      </c>
+      <c r="CK13" t="n">
+        <v>0.01415524560871515</v>
+      </c>
+      <c r="CL13" t="n">
+        <v>0.9364186972014641</v>
+      </c>
+      <c r="CM13" t="n">
+        <v>0.9371428571428572</v>
+      </c>
+      <c r="CN13" t="n">
+        <v>0.02025958966633972</v>
+      </c>
+      <c r="CO13" t="inlineStr">
+        <is>
+          <t>0.9425287356321839, 0.9111111111111111, 0.8913043478260869, 0.9540229885057471, 0.9101123595505618, 0.9111111111111111, 0.8602150537634409</t>
+        </is>
+      </c>
+      <c r="CP13" t="inlineStr">
+        <is>
+          <t>0.9913419913419913, 0.9868995633187773, 0.986784140969163, 0.9913793103448276, 0.9826086956521739, 0.9868995633187773, 0.9778761061946902</t>
+        </is>
+      </c>
+      <c r="CQ13" t="n">
+        <v>0.9862556244486288</v>
+      </c>
+      <c r="CR13" t="n">
+        <v>0.9868995633187773</v>
+      </c>
+      <c r="CS13" t="n">
+        <v>0.004419895690442677</v>
+      </c>
+      <c r="CT13" t="n">
+        <v>0.9114865296428919</v>
+      </c>
+      <c r="CU13" t="n">
+        <v>0.9111111111111111</v>
+      </c>
+      <c r="CV13" t="n">
+        <v>0.02881275463750477</v>
+      </c>
+      <c r="CW13" t="inlineStr">
+        <is>
+          <t>0.9761904761904762, 0.9647058823529412, 0.9647058823529412, 0.9764705882352941, 0.9529411764705882, 0.9647058823529412, 0.9411764705882353</t>
+        </is>
+      </c>
+      <c r="CX13" t="inlineStr">
+        <is>
+          <t>0.9786324786324786, 0.9658119658119658, 0.9572649572649573, 0.9829059829059829, 0.9658119658119658, 0.9658119658119658, 0.9444444444444444</t>
+        </is>
+      </c>
+      <c r="CY13" t="n">
+        <v>0.9658119658119658</v>
+      </c>
+      <c r="CZ13" t="n">
+        <v>0.9658119658119658</v>
+      </c>
+      <c r="DA13" t="n">
+        <v>0.01186948845862244</v>
+      </c>
+      <c r="DB13" t="n">
+        <v>0.9629851940776311</v>
+      </c>
+      <c r="DC13" t="n">
+        <v>0.9647058823529412</v>
+      </c>
+      <c r="DD13" t="n">
+        <v>0.01159815469077017</v>
+      </c>
+      <c r="DE13" t="inlineStr">
+        <is>
+          <t>0.9979649979649979, 0.9974358974358974, 0.9936400201106084, 0.9979135243841126, 0.993815987933635, 0.9961287078934138, 0.9934640522875816</t>
+        </is>
+      </c>
+      <c r="DF13" t="n">
+        <v>0.9957661697157495</v>
+      </c>
+      <c r="DG13" t="n">
+        <v>0.9961287078934138</v>
+      </c>
+      <c r="DH13" t="n">
+        <v>0.001926835603890327</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier_splashing_smote_grid-opt-mean-smote_default-model</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>{'estimator': 'RandomForestClassifier', 'estimator_params': {}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {'k_neighbors': 3, 'sampling_strategy': 0.9}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.9166666666666666</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.8799999999999999</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.9533179012345678</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.8101851851851851</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.8260869565217391</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.7037037037037037</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.9948186528497409</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>1</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0.9974025974025974</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0.9999751984126984</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0.996308954203691</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0.9952380952380953</v>
+      </c>
+      <c r="V14" t="n">
+        <v>1</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.9904761904761905</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0.9952153110047847</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>0.08466815948486328, 0.07819819450378418, 0.07041501998901367, 0.06761980056762695, 0.07537388801574707, 0.06524491310119629, 0.07358479499816895</t>
+        </is>
+      </c>
+      <c r="Z14" t="n">
+        <v>0.07358639580862862</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0.07358479499816895</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>0.006123812088318267</v>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>0.013681888580322266, 0.011255979537963867, 0.011024951934814453, 0.010769128799438477, 0.012682914733886719, 0.010698080062866211, 0.012078046798706055</t>
+        </is>
+      </c>
+      <c r="AD14" t="n">
+        <v>0.01174157006399972</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>0.01125597953796387</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>0.001038407807507469</v>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.8867924528301887, 0.8867924528301887, 0.8490566037735849, 0.9622641509433962, 0.8113207547169812, 0.8490566037735849</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>0.9210526315789473, 0.8738095238095238, 0.8769349845201238, 0.8475232198142415, 0.9473684210526316, 0.8297213622291022, 0.8243034055727554</t>
+        </is>
+      </c>
+      <c r="AI14" t="n">
+        <v>0.8743876497967608</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>0.8738095238095238</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0.04265449734207535</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>0.8842467804731956</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>0.8867924528301887</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>0.05002618177810771</v>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>0.958904109589041, 0.9142857142857143, 0.9117647058823528, 0.8787878787878787, 0.9714285714285714, 0.8387096774193549, 0.8857142857142858</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>0.9142857142857143, 0.8333333333333334, 0.8421052631578947, 0.8, 0.9444444444444444, 0.7727272727272727, 0.7777777777777778</t>
+        </is>
+      </c>
+      <c r="AQ14" t="n">
+        <v>0.8406676865323481</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>0.06149330978186609</v>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>0.9365949119373776, 0.8738095238095238, 0.8769349845201238, 0.8393939393939394, 0.9579365079365079, 0.8057184750733137, 0.8317460317460318</t>
+        </is>
+      </c>
+      <c r="AU14" t="n">
+        <v>0.8745906249166883</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>0.8738095238095238</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>0.05156828043059845</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>0.9085135633010285</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>0.9117647058823528</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>0.04279085169319258</v>
+      </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>0.9210526315789473, 0.9142857142857143, 0.9117647058823529, 0.90625, 0.9444444444444444, 0.9285714285714286, 0.8611111111111112</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>1.0, 0.8333333333333334, 0.8421052631578947, 0.7619047619047619, 1.0, 0.68, 0.8235294117647058</t>
+        </is>
+      </c>
+      <c r="BC14" t="n">
+        <v>0.8486961100229565</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>0.1086867495936684</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>0.9124971479819999</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>0.02401040141082343</v>
+      </c>
+      <c r="BI14" t="inlineStr">
+        <is>
+          <t>1.0, 0.9142857142857143, 0.9117647058823529, 0.8529411764705882, 1.0, 0.7647058823529411, 0.9117647058823529</t>
+        </is>
+      </c>
+      <c r="BJ14" t="inlineStr">
+        <is>
+          <t>0.8421052631578947, 0.8333333333333334, 0.8421052631578947, 0.8421052631578947, 0.8947368421052632, 0.8947368421052632, 0.7368421052631579</t>
+        </is>
+      </c>
+      <c r="BK14" t="n">
+        <v>0.8408521303258144</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>0.8421052631578947</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>0.04882395924505805</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>0.907923169267707</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>0.9117647058823529</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>0.0761206684010938</v>
+      </c>
+      <c r="BQ14" t="inlineStr">
+        <is>
+          <t>0.9969924812030075, 0.946031746031746, 0.976780185758514, 0.9342105263157895, 0.9512383900928792, 0.9195046439628484, 0.9411764705882354</t>
+        </is>
+      </c>
+      <c r="BR14" t="n">
+        <v>0.9522763491361458</v>
+      </c>
+      <c r="BS14" t="n">
+        <v>0.946031746031746</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>0.02438854772535699</v>
+      </c>
+      <c r="BU14" t="inlineStr">
+        <is>
+          <t>0.9968553459119497, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9968652037617555, 1.0, 0.9968652037617555</t>
+        </is>
+      </c>
+      <c r="BV14" t="inlineStr">
+        <is>
+          <t>0.995575221238938, 1.0, 0.995575221238938, 0.995575221238938, 0.995575221238938, 1.0, 0.995575221238938</t>
+        </is>
+      </c>
+      <c r="BW14" t="n">
+        <v>0.9968394437420985</v>
+      </c>
+      <c r="BX14" t="n">
+        <v>0.995575221238938</v>
+      </c>
+      <c r="BY14" t="n">
+        <v>0.001998911289613391</v>
+      </c>
+      <c r="BZ14" t="n">
+        <v>0.9977594515655674</v>
+      </c>
+      <c r="CA14" t="n">
+        <v>0.9968652037617555</v>
+      </c>
+      <c r="CB14" t="n">
+        <v>0.001417051170840857</v>
+      </c>
+      <c r="CC14" t="inlineStr">
+        <is>
+          <t>0.9975669099756691, 1.0, 0.9975786924939467, 0.9975786924939467, 0.9975786924939467, 1.0, 0.9975786924939467</t>
+        </is>
+      </c>
+      <c r="CD14" t="inlineStr">
+        <is>
+          <t>0.9955555555555555, 1.0, 0.9955555555555555, 0.9955555555555555, 0.9955555555555555, 1.0, 0.9955555555555555</t>
+        </is>
+      </c>
+      <c r="CE14" t="n">
+        <v>0.9968253968253968</v>
+      </c>
+      <c r="CF14" t="n">
+        <v>0.9955555555555555</v>
+      </c>
+      <c r="CG14" t="n">
+        <v>0.00200779533978946</v>
+      </c>
+      <c r="CH14" t="inlineStr">
+        <is>
+          <t>0.9965612327656124, 1.0, 0.9965671240247511, 0.9965671240247511, 0.9965671240247511, 1.0, 0.9965671240247511</t>
+        </is>
+      </c>
+      <c r="CI14" t="n">
+        <v>0.9975471041235167</v>
+      </c>
+      <c r="CJ14" t="n">
+        <v>0.9965671240247511</v>
+      </c>
+      <c r="CK14" t="n">
+        <v>0.001551348844990803</v>
+      </c>
+      <c r="CL14" t="n">
+        <v>0.9982688114216364</v>
+      </c>
+      <c r="CM14" t="n">
+        <v>0.9975786924939467</v>
+      </c>
+      <c r="CN14" t="n">
+        <v>0.001094907038779773</v>
+      </c>
+      <c r="CO14" t="inlineStr">
+        <is>
+          <t>0.9951456310679612, 1.0, 0.9951690821256038, 0.9951690821256038, 0.9951690821256038, 1.0, 0.9951690821256038</t>
+        </is>
+      </c>
+      <c r="CP14" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CQ14" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR14" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS14" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT14" t="n">
+        <v>0.9965459942243395</v>
+      </c>
+      <c r="CU14" t="n">
+        <v>0.9951690821256038</v>
+      </c>
+      <c r="CV14" t="n">
+        <v>0.002184519446236978</v>
+      </c>
+      <c r="CW14" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CX14" t="inlineStr">
+        <is>
+          <t>0.9911504424778761, 1.0, 0.9911504424778761, 0.9911504424778761, 0.9911504424778761, 1.0, 0.9911504424778761</t>
+        </is>
+      </c>
+      <c r="CY14" t="n">
+        <v>0.9936788874841972</v>
+      </c>
+      <c r="CZ14" t="n">
+        <v>0.9911504424778761</v>
+      </c>
+      <c r="DA14" t="n">
+        <v>0.003997822579226782</v>
+      </c>
+      <c r="DB14" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC14" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD14" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE14" t="inlineStr">
+        <is>
+          <t>0.9999784157133607, 1.0, 0.9999785204914512, 0.9999785204914512, 0.9999785204914512, 1.0, 0.9999785204914511</t>
+        </is>
+      </c>
+      <c r="DF14" t="n">
+        <v>0.999984642525595</v>
+      </c>
+      <c r="DG14" t="n">
+        <v>0.9999785204914512</v>
+      </c>
+      <c r="DH14" t="n">
+        <v>9.712984233453662e-06</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier_no_fragmentation_smote_grid-opt-mean-smote_default-model</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>{'estimator': 'RandomForestClassifier', 'estimator_params': {}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {'k_neighbors': 8, 'sampling_strategy': 0.9}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0.9066666666666666</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.7826086956521739</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.8372093023255814</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.9777272727272727</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.8858943707889591</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.9045454545454545</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.9615384615384616</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.9345794392523366</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" t="n">
+        <v>1</v>
+      </c>
+      <c r="T15" t="n">
+        <v>1</v>
+      </c>
+      <c r="U15" t="n">
+        <v>1</v>
+      </c>
+      <c r="V15" t="n">
+        <v>1</v>
+      </c>
+      <c r="W15" t="n">
+        <v>1</v>
+      </c>
+      <c r="X15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>0.10165286064147949, 0.07521605491638184, 0.0776362419128418, 0.07327508926391602, 0.07524776458740234, 0.07541704177856445, 0.0753777027130127</t>
+        </is>
+      </c>
+      <c r="Z15" t="n">
+        <v>0.0791175365447998</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0.0753777027130127</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>0.009273972555047529</v>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>0.012701988220214844, 0.011260986328125, 0.011708974838256836, 0.010669946670532227, 0.01034402847290039, 0.009556055068969727, 0.011501073837280273</t>
+        </is>
+      </c>
+      <c r="AD15" t="n">
+        <v>0.01110615049089704</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>0.011260986328125</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>0.0009459638620693968</v>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>0.8333333333333334, 0.8113207547169812, 0.9056603773584906, 0.8113207547169812, 0.9433962264150944, 0.9056603773584906, 0.9245283018867925</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>0.782051282051282, 0.7802197802197802, 0.8672161172161172, 0.8031135531135531, 0.9386446886446886, 0.8901098901098901, 0.9258241758241759</t>
+        </is>
+      </c>
+      <c r="AI15" t="n">
+        <v>0.8553113553113555</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>0.8672161172161172</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0.06210539109258142</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>0.8764600179694518</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>0.9056603773584906</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>0.05188241659008128</v>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>0.689655172413793, 0.6666666666666666, 0.8148148148148148, 0.6875000000000001, 0.896551724137931, 0.8275862068965518, 0.8666666666666666</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>0.8860759493670887, 0.868421052631579, 0.9367088607594937, 0.8648648648648648, 0.9610389610389611, 0.935064935064935, 0.9473684210526315</t>
+        </is>
+      </c>
+      <c r="AQ15" t="n">
+        <v>0.9142204349685078</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>0.935064935064935</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>0.03694910328727866</v>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>0.7878655608904408, 0.7675438596491229, 0.8757618377871542, 0.7761824324324325, 0.9287953425884461, 0.8813255709807435, 0.9070175438596491</t>
+        </is>
+      </c>
+      <c r="AU15" t="n">
+        <v>0.8463560211697126</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>0.8757618377871542</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>0.06224428467103883</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>0.7784916073709177</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>0.8148148148148148</v>
+      </c>
+      <c r="AZ15" t="n">
+        <v>0.08792764030382219</v>
+      </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>0.7142857142857143, 0.625, 0.8461538461538461, 0.6111111111111112, 0.8666666666666667, 0.8, 0.8125</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>0.875, 0.8918918918918919, 0.925, 0.9142857142857143, 0.9736842105263158, 0.9473684210526315, 0.972972972972973</t>
+        </is>
+      </c>
+      <c r="BC15" t="n">
+        <v>0.9286004586756466</v>
+      </c>
+      <c r="BD15" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="BE15" t="n">
+        <v>0.03544030065368339</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>0.7536739054596199</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>0.09662820782542658</v>
+      </c>
+      <c r="BI15" t="inlineStr">
+        <is>
+          <t>0.6666666666666666, 0.7142857142857143, 0.7857142857142857, 0.7857142857142857, 0.9285714285714286, 0.8571428571428571, 0.9285714285714286</t>
+        </is>
+      </c>
+      <c r="BJ15" t="inlineStr">
+        <is>
+          <t>0.8974358974358975, 0.8461538461538461, 0.9487179487179487, 0.8205128205128205, 0.9487179487179487, 0.9230769230769231, 0.9230769230769231</t>
+        </is>
+      </c>
+      <c r="BK15" t="n">
+        <v>0.9010989010989012</v>
+      </c>
+      <c r="BL15" t="n">
+        <v>0.9230769230769231</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>0.04633373861052571</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>0.8095238095238094</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>0.09352195295828246</v>
+      </c>
+      <c r="BQ15" t="inlineStr">
+        <is>
+          <t>0.9324786324786324, 0.8763736263736264, 0.9752747252747253, 0.9130036630036629, 0.9945054945054945, 0.9313186813186813, 0.989010989010989</t>
+        </is>
+      </c>
+      <c r="BR15" t="n">
+        <v>0.9445665445665447</v>
+      </c>
+      <c r="BS15" t="n">
+        <v>0.9324786324786324</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>0.04032070154024791</v>
+      </c>
+      <c r="BU15" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BV15" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BW15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY15" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC15" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CD15" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CE15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH15" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CI15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO15" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CP15" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CQ15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CU15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV15" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW15" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CX15" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CY15" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ15" t="n">
+        <v>1</v>
+      </c>
+      <c r="DA15" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB15" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC15" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD15" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE15" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="DF15" t="n">
+        <v>1</v>
+      </c>
+      <c r="DG15" t="n">
+        <v>1</v>
+      </c>
+      <c r="DH15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>splashing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>LGBMClassifier_splashing_smote_grid-opt-mean-smote_default-model</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>{'estimator': 'LGBMClassifier', 'estimator_params': {'verbose': -1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': ('inclination', 'volume_fraction'), 'passthrough_features': ('wettability',), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {'k_neighbors': 10, 'sampling_strategy': 1.0}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.8679245283018868</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.910891089108911</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.9506172839506173</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.863608809860578</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.849537037037037</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.7407407407407407</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.8163265306122449</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.9966329966329966</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0.9948186528497409</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0.9974025974025974</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0.9999751984126984</v>
+      </c>
+      <c r="T16" t="n">
+        <v>0.996308954203691</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0.9952380952380953</v>
+      </c>
+      <c r="V16" t="n">
+        <v>1</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.9904761904761905</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0.9952153110047847</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>0.46227097511291504, 0.48512792587280273, 0.4832901954650879, 0.4716978073120117, 0.45341992378234863, 0.5346879959106445, 0.48238706588745117</t>
+        </is>
+      </c>
+      <c r="Z16" t="n">
+        <v>0.4818402699061802</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.4823870658874512</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0.02420045753861314</v>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>0.01100921630859375, 0.012105941772460938, 0.010255813598632812, 0.010008096694946289, 0.009479999542236328, 0.009672880172729492, 0.009705066680908203</t>
+        </is>
+      </c>
+      <c r="AD16" t="n">
+        <v>0.01031957353864397</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>0.01000809669494629</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>0.0008675513368268544</v>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>0.9629629629629629, 0.8301886792452831, 0.9433962264150944, 0.8679245283018868, 0.9056603773584906, 0.8679245283018868, 0.8867924528301887</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>0.9473684210526316, 0.830952380952381, 0.9326625386996904, 0.8854489164086687, 0.903250773993808, 0.8854489164086687, 0.8885448916408669</t>
+        </is>
+      </c>
+      <c r="AI16" t="n">
+        <v>0.8962395484509594</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>0.8885448916408669</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0.03493759861513632</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>0.8949785364879705</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>0.8867924528301887</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>0.04277655056961074</v>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>0.9722222222222222, 0.8656716417910447, 0.9565217391304348, 0.888888888888889, 0.9253731343283583, 0.888888888888889, 0.9090909090909091</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>0.9444444444444444, 0.7692307692307692, 0.918918918918919, 0.8372093023255814, 0.8717948717948718, 0.8372093023255814, 0.8500000000000001</t>
+        </is>
+      </c>
+      <c r="AQ16" t="n">
+        <v>0.8612582298628809</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>0.8500000000000001</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>0.0535966753545923</v>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>0.9583333333333333, 0.8174512055109069, 0.937720329024677, 0.8630490956072352, 0.898584003061615, 0.8630490956072352, 0.8795454545454546</t>
+        </is>
+      </c>
+      <c r="AU16" t="n">
+        <v>0.888247502384351</v>
+      </c>
+      <c r="AV16" t="n">
+        <v>0.8795454545454546</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>0.04443966731526079</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>0.9152367749058211</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="AZ16" t="n">
+        <v>0.03573200154652034</v>
+      </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>0.9459459459459459, 0.90625, 0.9428571428571428, 0.9655172413793104, 0.9393939393939394, 0.9655172413793104, 0.9375</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>1.0, 0.7142857142857143, 0.9444444444444444, 0.75, 0.85, 0.75, 0.8095238095238095</t>
+        </is>
+      </c>
+      <c r="BC16" t="n">
+        <v>0.8311791383219954</v>
+      </c>
+      <c r="BD16" t="n">
+        <v>0.8095238095238095</v>
+      </c>
+      <c r="BE16" t="n">
+        <v>0.09928089198165066</v>
+      </c>
+      <c r="BF16" t="n">
+        <v>0.9432830729936642</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>0.9428571428571428</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>0.01857804612671459</v>
+      </c>
+      <c r="BI16" t="inlineStr">
+        <is>
+          <t>1.0, 0.8285714285714286, 0.9705882352941176, 0.8235294117647058, 0.9117647058823529, 0.8235294117647058, 0.8823529411764706</t>
+        </is>
+      </c>
+      <c r="BJ16" t="inlineStr">
+        <is>
+          <t>0.8947368421052632, 0.8333333333333334, 0.8947368421052632, 0.9473684210526315, 0.8947368421052632, 0.9473684210526315, 0.8947368421052632</t>
+        </is>
+      </c>
+      <c r="BK16" t="n">
+        <v>0.9010025062656641</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>0.03592799796198356</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>0.8914765906362546</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>0.8823529411764706</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>0.067317508811085</v>
+      </c>
+      <c r="BQ16" t="inlineStr">
+        <is>
+          <t>0.9924812030075187, 0.9365079365079365, 0.9876160990712075, 0.9705882352941176, 0.958204334365325, 0.9125386996904025, 0.9380804953560371</t>
+        </is>
+      </c>
+      <c r="BR16" t="n">
+        <v>0.9565738576132208</v>
+      </c>
+      <c r="BS16" t="n">
+        <v>0.958204334365325</v>
+      </c>
+      <c r="BT16" t="n">
+        <v>0.02708652858338519</v>
+      </c>
+      <c r="BU16" t="inlineStr">
+        <is>
+          <t>0.9968553459119497, 1.0, 0.9968652037617555, 0.9968652037617555, 0.9968652037617555, 1.0, 0.9968652037617555</t>
+        </is>
+      </c>
+      <c r="BV16" t="inlineStr">
+        <is>
+          <t>0.995575221238938, 1.0, 0.995575221238938, 0.995575221238938, 0.995575221238938, 1.0, 0.995575221238938</t>
+        </is>
+      </c>
+      <c r="BW16" t="n">
+        <v>0.9968394437420985</v>
+      </c>
+      <c r="BX16" t="n">
+        <v>0.995575221238938</v>
+      </c>
+      <c r="BY16" t="n">
+        <v>0.001998911289613391</v>
+      </c>
+      <c r="BZ16" t="n">
+        <v>0.9977594515655674</v>
+      </c>
+      <c r="CA16" t="n">
+        <v>0.9968652037617555</v>
+      </c>
+      <c r="CB16" t="n">
+        <v>0.001417051170840857</v>
+      </c>
+      <c r="CC16" t="inlineStr">
+        <is>
+          <t>0.9975669099756691, 1.0, 0.9975786924939467, 0.9975786924939467, 0.9975786924939467, 1.0, 0.9975786924939467</t>
+        </is>
+      </c>
+      <c r="CD16" t="inlineStr">
+        <is>
+          <t>0.9955555555555555, 1.0, 0.9955555555555555, 0.9955555555555555, 0.9955555555555555, 1.0, 0.9955555555555555</t>
+        </is>
+      </c>
+      <c r="CE16" t="n">
+        <v>0.9968253968253968</v>
+      </c>
+      <c r="CF16" t="n">
+        <v>0.9955555555555555</v>
+      </c>
+      <c r="CG16" t="n">
+        <v>0.00200779533978946</v>
+      </c>
+      <c r="CH16" t="inlineStr">
+        <is>
+          <t>0.9965612327656124, 1.0, 0.9965671240247511, 0.9965671240247511, 0.9965671240247511, 1.0, 0.9965671240247511</t>
+        </is>
+      </c>
+      <c r="CI16" t="n">
+        <v>0.9975471041235167</v>
+      </c>
+      <c r="CJ16" t="n">
+        <v>0.9965671240247511</v>
+      </c>
+      <c r="CK16" t="n">
+        <v>0.001551348844990803</v>
+      </c>
+      <c r="CL16" t="n">
+        <v>0.9982688114216364</v>
+      </c>
+      <c r="CM16" t="n">
+        <v>0.9975786924939467</v>
+      </c>
+      <c r="CN16" t="n">
+        <v>0.001094907038779773</v>
+      </c>
+      <c r="CO16" t="inlineStr">
+        <is>
+          <t>0.9951456310679612, 1.0, 0.9951690821256038, 0.9951690821256038, 0.9951690821256038, 1.0, 0.9951690821256038</t>
+        </is>
+      </c>
+      <c r="CP16" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CQ16" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR16" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS16" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT16" t="n">
+        <v>0.9965459942243395</v>
+      </c>
+      <c r="CU16" t="n">
+        <v>0.9951690821256038</v>
+      </c>
+      <c r="CV16" t="n">
+        <v>0.002184519446236978</v>
+      </c>
+      <c r="CW16" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CX16" t="inlineStr">
+        <is>
+          <t>0.9911504424778761, 1.0, 0.9911504424778761, 0.9911504424778761, 0.9911504424778761, 1.0, 0.9911504424778761</t>
+        </is>
+      </c>
+      <c r="CY16" t="n">
+        <v>0.9936788874841972</v>
+      </c>
+      <c r="CZ16" t="n">
+        <v>0.9911504424778761</v>
+      </c>
+      <c r="DA16" t="n">
+        <v>0.003997822579226782</v>
+      </c>
+      <c r="DB16" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC16" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE16" t="inlineStr">
+        <is>
+          <t>0.9999784157133607, 1.0, 0.9999785204914511, 0.9999785204914512, 0.9999785204914512, 1.0, 0.9999785204914511</t>
+        </is>
+      </c>
+      <c r="DF16" t="n">
+        <v>0.999984642525595</v>
+      </c>
+      <c r="DG16" t="n">
+        <v>0.9999785204914512</v>
+      </c>
+      <c r="DH16" t="n">
+        <v>9.712984233463661e-06</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>df_dimless</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>no_fragmentation</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>LGBMClassifier_no_fragmentation_smote_grid-opt-mean-smote_default-model</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>{'estimator': 'LGBMClassifier', 'estimator_params': {'verbose': -1}, 'source_features': ('init_volume_fraction', 'volume_fraction', 'sedimentation_Re', 'sign_sedimentation_Re', 'sign_sedimentation_Stk', 'sedimentation_Stk', 'particle_liquid_density_ratio', 'particle_droplet_diameter_ratio', 'sign_particle_droplet_diameter_ratio', 'wettability', 'relative_roughness', 'inclination', 'Re', 'We', 'K'), 'features_to_drop': ('Re', 'We', 'init_volume_fraction', 'particle_liquid_density_ratio', 'sedimentation_Re', 'sign_particle_droplet_diameter_ratio', 'sign_sedimentation_Re', 'sign_sedimentation_Stk'), 'log_features': ('relative_roughness', 'sedimentation_Stk', 'particle_droplet_diameter_ratio'), 'minmax_features': (), 'passthrough_features': ('wettability', 'inclination', 'volume_fraction'), 'std_features': ('sedimentation_Stk', 'particle_droplet_diameter_ratio', 'relative_roughness', 'K'), 'add_init_transformer': True, 'add_df_transformer': True, 'add_const': False, 'add_smote': True, 'is_smotenc': False, 'smote_params': {'k_neighbors': 3, 'sampling_strategy': 0.9}, 'random_state': 42}</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0.9066666666666666</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.7826086956521739</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.8372093023255814</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.980909090909091</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.8858943707889591</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.9045454545454545</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.9615384615384616</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.9345794392523366</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" t="n">
+        <v>1</v>
+      </c>
+      <c r="U17" t="n">
+        <v>1</v>
+      </c>
+      <c r="V17" t="n">
+        <v>1</v>
+      </c>
+      <c r="W17" t="n">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>0.57930588722229, 0.5847277641296387, 0.49130702018737793, 0.4850151538848877, 0.4905588626861572, 0.5041279792785645, 0.5337998867034912</t>
+        </is>
+      </c>
+      <c r="Z17" t="n">
+        <v>0.5241203648703439</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>0.5041279792785645</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0.03954092796649499</v>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>0.00900721549987793, 0.00811314582824707, 0.008222103118896484, 0.008510828018188477, 0.008167028427124023, 0.008897781372070312, 0.008836984634399414</t>
+        </is>
+      </c>
+      <c r="AD17" t="n">
+        <v>0.008536440985543388</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0.008510828018188477</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>0.000350026682689712</v>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>0.9074074074074074, 0.8679245283018868, 0.9056603773584906, 0.8679245283018868, 0.9433962264150944, 0.9245283018867925, 0.9245283018867925</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>0.8333333333333333, 0.8644688644688645, 0.8672161172161172, 0.8644688644688645, 0.9157509157509157, 0.9029304029304028, 0.9258241758241759</t>
+        </is>
+      </c>
+      <c r="AI17" t="n">
+        <v>0.8819989534275249</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>0.8672161172161172</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>0.03093646373846525</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>0.9059099530797645</v>
+      </c>
+      <c r="AM17" t="n">
+        <v>0.9074074074074074</v>
+      </c>
+      <c r="AN17" t="n">
+        <v>0.02669027688607385</v>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>0.8, 0.7741935483870968, 0.8148148148148148, 0.7741935483870968, 0.888888888888889, 0.8571428571428571, 0.8666666666666666</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>0.9397590361445783, 0.9066666666666667, 0.9367088607594937, 0.9066666666666667, 0.9620253164556962, 0.9487179487179487, 0.9473684210526315</t>
+        </is>
+      </c>
+      <c r="AQ17" t="n">
+        <v>0.9354161309233833</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>0.9397590361445783</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>0.01964484562333443</v>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>0.8698795180722891, 0.8404301075268817, 0.8757618377871542, 0.8404301075268817, 0.9254571026722926, 0.9029304029304028, 0.9070175438596491</t>
+        </is>
+      </c>
+      <c r="AU17" t="n">
+        <v>0.8802723743393643</v>
+      </c>
+      <c r="AV17" t="n">
+        <v>0.8757618377871542</v>
+      </c>
+      <c r="AW17" t="n">
+        <v>0.03064431636352031</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>0.8251286177553459</v>
+      </c>
+      <c r="AY17" t="n">
+        <v>0.8148148148148148</v>
+      </c>
+      <c r="AZ17" t="n">
+        <v>0.04266527150878797</v>
+      </c>
+      <c r="BA17" t="inlineStr">
+        <is>
+          <t>1.0, 0.7058823529411765, 0.8461538461538461, 0.7058823529411765, 0.9230769230769231, 0.8571428571428571, 0.8125</t>
+        </is>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>0.8863636363636364, 0.9444444444444444, 0.925, 0.9444444444444444, 0.95, 0.9487179487179487, 0.972972972972973</t>
+        </is>
+      </c>
+      <c r="BC17" t="n">
+        <v>0.938849063849064</v>
+      </c>
+      <c r="BD17" t="n">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="BE17" t="n">
+        <v>0.02505796900711914</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>0.8358054760365684</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>0.09960041652786275</v>
+      </c>
+      <c r="BI17" t="inlineStr">
+        <is>
+          <t>0.6666666666666666, 0.8571428571428571, 0.7857142857142857, 0.8571428571428571, 0.8571428571428571, 0.8571428571428571, 0.9285714285714286</t>
+        </is>
+      </c>
+      <c r="BJ17" t="inlineStr">
+        <is>
+          <t>1.0, 0.8717948717948718, 0.9487179487179487, 0.8717948717948718, 0.9743589743589743, 0.9487179487179487, 0.9230769230769231</t>
+        </is>
+      </c>
+      <c r="BK17" t="n">
+        <v>0.9340659340659341</v>
+      </c>
+      <c r="BL17" t="n">
+        <v>0.9487179487179487</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>0.04516054214629286</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>0.8299319727891156</v>
+      </c>
+      <c r="BO17" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>0.07681353599072255</v>
+      </c>
+      <c r="BQ17" t="inlineStr">
+        <is>
+          <t>0.958974358974359, 0.9157509157509158, 0.9835164835164836, 0.9377289377289377, 0.9835164835164836, 0.9065934065934067, 0.9908424908424909</t>
+        </is>
+      </c>
+      <c r="BR17" t="n">
+        <v>0.9538461538461539</v>
+      </c>
+      <c r="BS17" t="n">
+        <v>0.958974358974359</v>
+      </c>
+      <c r="BT17" t="n">
+        <v>0.03184677222556585</v>
+      </c>
+      <c r="BU17" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BV17" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="BW17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BX17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BY17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC17" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CD17" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CE17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH17" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CI17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO17" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CP17" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CQ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CU17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV17" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW17" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CX17" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="CY17" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ17" t="n">
+        <v>1</v>
+      </c>
+      <c r="DA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB17" t="n">
+        <v>1</v>
+      </c>
+      <c r="DC17" t="n">
+        <v>1</v>
+      </c>
+      <c r="DD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="DE17" t="inlineStr">
+        <is>
+          <t>1.0, 1.0, 1.0, 1.0, 1.0, 1.0, 1.0</t>
+        </is>
+      </c>
+      <c r="DF17" t="n">
+        <v>1</v>
+      </c>
+      <c r="DG17" t="n">
+        <v>1</v>
+      </c>
+      <c r="DH17" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>